<commit_message>
precios por excel update
</commit_message>
<xml_diff>
--- a/app/public/templates/precios.xlsx
+++ b/app/public/templates/precios.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28623"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DataFlow\app\public\templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{604A8015-66F4-431E-A348-0E5B55E651C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Hoja1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -58,10 +52,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.00000"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -73,10 +65,9 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -87,7 +78,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -100,21 +98,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -125,10 +124,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -166,71 +165,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -258,7 +257,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -281,11 +280,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -294,13 +293,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -310,7 +309,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -319,7 +318,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -328,7 +327,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -336,10 +335,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -404,23 +403,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="2" width="23.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="2" width="21.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="2" width="29.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="2" width="29.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="2" width="13.719285714285713" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -451,7 +454,7 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
arreglos finales actualizador listp por excel
</commit_message>
<xml_diff>
--- a/app/public/templates/precios.xlsx
+++ b/app/public/templates/precios.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Hoja1"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Lista de Precios - Cód.</t>
   </si>
@@ -47,13 +47,15 @@
   </si>
   <si>
     <t>Precio</t>
+  </si>
+  <si>
+    <t>Moneda</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -97,23 +99,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -124,10 +127,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -165,71 +168,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -257,7 +260,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -280,11 +283,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -293,13 +296,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -309,7 +312,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -318,7 +321,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -327,7 +330,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -335,10 +338,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -407,23 +410,19 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="23.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="21.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="2" width="29.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="2" width="29.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="2" width="13.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="1" max="3" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row r="1" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -454,7 +453,10 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
arreglos generales & sesiones manager
</commit_message>
<xml_diff>
--- a/app/public/templates/precios.xlsx
+++ b/app/public/templates/precios.xlsx
@@ -2,14 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508"/>
+    <workbookView xWindow="192" yWindow="60" windowWidth="22116" windowHeight="9288"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
@@ -46,30 +48,23 @@
     <t>Artículo - Elemento 3</t>
   </si>
   <si>
+    <t>Moneda</t>
+  </si>
+  <si>
     <t>Precio</t>
-  </si>
-  <si>
-    <t>Moneda</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -80,14 +75,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -99,21 +87,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -123,7 +104,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -133,28 +114,28 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="0000FF"/>
@@ -256,6 +237,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
@@ -266,31 +248,31 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="51000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
+                <a:shade val="93000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="94000"/>
+                <a:shade val="94000"/>
                 <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="9500"/>
+              <a:shade val="95000"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -312,7 +294,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -370,7 +352,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="20000"/>
+                <a:shade val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -383,12 +365,13 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
                 <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
+                <a:shade val="30000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -407,60 +390,66 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-  </sheetPr>
   <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="3" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
         <v>11</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>